<commit_message>
Add worker schedule excel.
</commit_message>
<xml_diff>
--- a/schedule_with_image.xlsx
+++ b/schedule_with_image.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="schedule_shifts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="shift_schedule" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="worker_schedule" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -181,6 +182,36 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1428750" cy="190500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1914,4 +1945,2184 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A3:AQ23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="12" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
+    <col width="12" customWidth="1" min="39" max="39"/>
+    <col width="12" customWidth="1" min="40" max="40"/>
+    <col width="12" customWidth="1" min="41" max="41"/>
+    <col width="12" customWidth="1" min="42" max="42"/>
+    <col width="12" customWidth="1" min="43" max="43"/>
+  </cols>
+  <sheetData>
+    <row r="3">
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>23/09/2024</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>24/09/2024</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>25/09/2024</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>26/09/2024</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>27/09/2024</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>28/09/2024</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>29/09/2024</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>30/09/2024</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>01/10/2024</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>02/10/2024</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>03/10/2024</t>
+        </is>
+      </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t>04/10/2024</t>
+        </is>
+      </c>
+      <c r="N3" s="1" t="inlineStr">
+        <is>
+          <t>05/10/2024</t>
+        </is>
+      </c>
+      <c r="O3" s="1" t="inlineStr">
+        <is>
+          <t>06/10/2024</t>
+        </is>
+      </c>
+      <c r="P3" s="1" t="inlineStr">
+        <is>
+          <t>07/10/2024</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>08/10/2024</t>
+        </is>
+      </c>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>09/10/2024</t>
+        </is>
+      </c>
+      <c r="S3" s="1" t="inlineStr">
+        <is>
+          <t>10/10/2024</t>
+        </is>
+      </c>
+      <c r="T3" s="1" t="inlineStr">
+        <is>
+          <t>11/10/2024</t>
+        </is>
+      </c>
+      <c r="U3" s="1" t="inlineStr">
+        <is>
+          <t>12/10/2024</t>
+        </is>
+      </c>
+      <c r="V3" s="1" t="inlineStr">
+        <is>
+          <t>13/10/2024</t>
+        </is>
+      </c>
+      <c r="W3" s="1" t="inlineStr">
+        <is>
+          <t>14/10/2024</t>
+        </is>
+      </c>
+      <c r="X3" s="1" t="inlineStr">
+        <is>
+          <t>15/10/2024</t>
+        </is>
+      </c>
+      <c r="Y3" s="1" t="inlineStr">
+        <is>
+          <t>16/10/2024</t>
+        </is>
+      </c>
+      <c r="Z3" s="1" t="inlineStr">
+        <is>
+          <t>17/10/2024</t>
+        </is>
+      </c>
+      <c r="AA3" s="1" t="inlineStr">
+        <is>
+          <t>18/10/2024</t>
+        </is>
+      </c>
+      <c r="AB3" s="1" t="inlineStr">
+        <is>
+          <t>19/10/2024</t>
+        </is>
+      </c>
+      <c r="AC3" s="1" t="inlineStr">
+        <is>
+          <t>20/10/2024</t>
+        </is>
+      </c>
+      <c r="AD3" s="1" t="inlineStr">
+        <is>
+          <t>21/10/2024</t>
+        </is>
+      </c>
+      <c r="AE3" s="1" t="inlineStr">
+        <is>
+          <t>22/10/2024</t>
+        </is>
+      </c>
+      <c r="AF3" s="1" t="inlineStr">
+        <is>
+          <t>23/10/2024</t>
+        </is>
+      </c>
+      <c r="AG3" s="1" t="inlineStr">
+        <is>
+          <t>24/10/2024</t>
+        </is>
+      </c>
+      <c r="AH3" s="1" t="inlineStr">
+        <is>
+          <t>25/10/2024</t>
+        </is>
+      </c>
+      <c r="AI3" s="1" t="inlineStr">
+        <is>
+          <t>26/10/2024</t>
+        </is>
+      </c>
+      <c r="AJ3" s="1" t="inlineStr">
+        <is>
+          <t>27/10/2024</t>
+        </is>
+      </c>
+      <c r="AK3" s="1" t="inlineStr">
+        <is>
+          <t>28/10/2024</t>
+        </is>
+      </c>
+      <c r="AL3" s="1" t="inlineStr">
+        <is>
+          <t>29/10/2024</t>
+        </is>
+      </c>
+      <c r="AM3" s="1" t="inlineStr">
+        <is>
+          <t>30/10/2024</t>
+        </is>
+      </c>
+      <c r="AN3" s="1" t="inlineStr">
+        <is>
+          <t>31/10/2024</t>
+        </is>
+      </c>
+      <c r="AO3" s="1" t="inlineStr">
+        <is>
+          <t>01/11/2024</t>
+        </is>
+      </c>
+      <c r="AP3" s="1" t="inlineStr">
+        <is>
+          <t>02/11/2024</t>
+        </is>
+      </c>
+      <c r="AQ3" s="1" t="inlineStr">
+        <is>
+          <t>03/11/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="AA4" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AC4" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="n"/>
+      <c r="R5" s="4" t="n"/>
+      <c r="S5" s="4" t="n"/>
+      <c r="T5" s="4" t="n"/>
+      <c r="U5" s="4" t="n"/>
+      <c r="V5" s="4" t="n"/>
+      <c r="W5" s="4" t="n"/>
+      <c r="X5" s="4" t="n"/>
+      <c r="Y5" s="4" t="n"/>
+      <c r="Z5" s="4" t="n"/>
+      <c r="AA5" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AB5" s="4" t="n"/>
+      <c r="AC5" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AD5" s="4" t="n"/>
+      <c r="AE5" s="4" t="n"/>
+      <c r="AF5" s="4" t="n"/>
+      <c r="AG5" s="4" t="n"/>
+      <c r="AH5" s="4" t="n"/>
+      <c r="AI5" s="4" t="n"/>
+      <c r="AJ5" s="4" t="n"/>
+      <c r="AK5" s="4" t="n"/>
+      <c r="AL5" s="4" t="n"/>
+      <c r="AM5" s="4" t="n"/>
+      <c r="AN5" s="4" t="n"/>
+      <c r="AO5" s="4" t="n"/>
+      <c r="AP5" s="4" t="n"/>
+      <c r="AQ5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>George</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="V6" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="X6" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AD6" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AF6" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AM6" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AN6" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="4" t="n"/>
+      <c r="C7" s="4" t="n"/>
+      <c r="D7" s="4" t="n"/>
+      <c r="E7" s="4" t="n"/>
+      <c r="F7" s="4" t="n"/>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="4" t="n"/>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="n"/>
+      <c r="R7" s="4" t="n"/>
+      <c r="S7" s="4" t="n"/>
+      <c r="T7" s="4" t="n"/>
+      <c r="U7" s="4" t="n"/>
+      <c r="V7" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="W7" s="4" t="n"/>
+      <c r="X7" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="Y7" s="4" t="n"/>
+      <c r="Z7" s="4" t="n"/>
+      <c r="AA7" s="4" t="n"/>
+      <c r="AB7" s="4" t="n"/>
+      <c r="AC7" s="4" t="n"/>
+      <c r="AD7" s="4" t="n"/>
+      <c r="AE7" s="4" t="n"/>
+      <c r="AF7" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AG7" s="4" t="n"/>
+      <c r="AH7" s="4" t="n"/>
+      <c r="AI7" s="4" t="n"/>
+      <c r="AJ7" s="4" t="n"/>
+      <c r="AK7" s="4" t="n"/>
+      <c r="AL7" s="4" t="n"/>
+      <c r="AM7" s="4" t="n"/>
+      <c r="AN7" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AO7" s="4" t="n"/>
+      <c r="AP7" s="4" t="n"/>
+      <c r="AQ7" s="4" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Linda</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="R8" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="Y8" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AD8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AE8" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AF8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AG8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AI8" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AK8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AL8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AM8" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AO8" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AP8" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="n"/>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4" t="n"/>
+      <c r="Q9" s="4" t="n"/>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="S9" s="4" t="n"/>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="U9" s="4" t="n"/>
+      <c r="V9" s="4" t="n"/>
+      <c r="W9" s="4" t="n"/>
+      <c r="X9" s="4" t="n"/>
+      <c r="Y9" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="Z9" s="4" t="n"/>
+      <c r="AA9" s="4" t="n"/>
+      <c r="AB9" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AC9" s="4" t="n"/>
+      <c r="AD9" s="4" t="n"/>
+      <c r="AE9" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AF9" s="4" t="n"/>
+      <c r="AG9" s="4" t="n"/>
+      <c r="AH9" s="4" t="n"/>
+      <c r="AI9" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AJ9" s="4" t="n"/>
+      <c r="AK9" s="4" t="n"/>
+      <c r="AL9" s="4" t="n"/>
+      <c r="AM9" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AN9" s="4" t="n"/>
+      <c r="AO9" s="4" t="n"/>
+      <c r="AP9" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AQ9" s="4" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Pattie</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="R10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="S10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="W10" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="X10" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="Y10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="Z10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AA10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AD10" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AE10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AF10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AG10" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AH10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AK10" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AM10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AN10" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AO10" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="n"/>
+      <c r="B11" s="4" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="n"/>
+      <c r="P11" s="4" t="n"/>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="n"/>
+      <c r="S11" s="4" t="n"/>
+      <c r="T11" s="4" t="n"/>
+      <c r="U11" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="V11" s="4" t="n"/>
+      <c r="W11" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="X11" s="4" t="n"/>
+      <c r="Y11" s="4" t="n"/>
+      <c r="Z11" s="4" t="n"/>
+      <c r="AA11" s="4" t="n"/>
+      <c r="AB11" s="4" t="n"/>
+      <c r="AC11" s="4" t="n"/>
+      <c r="AD11" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AE11" s="4" t="n"/>
+      <c r="AF11" s="4" t="n"/>
+      <c r="AG11" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AH11" s="4" t="n"/>
+      <c r="AI11" s="4" t="n"/>
+      <c r="AJ11" s="4" t="n"/>
+      <c r="AK11" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AL11" s="4" t="n"/>
+      <c r="AM11" s="4" t="n"/>
+      <c r="AN11" s="4" t="n"/>
+      <c r="AO11" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AP11" s="4" t="n"/>
+      <c r="AQ11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Vanessa</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="X12" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="Y12" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="Z12" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AA12" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AD12" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AF12" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AH12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AJ12" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AL12" s="5" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AQ12" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="4" t="n"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n"/>
+      <c r="E13" s="4" t="n"/>
+      <c r="F13" s="4" t="n"/>
+      <c r="G13" s="4" t="n"/>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="n"/>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="n"/>
+      <c r="O13" s="4" t="n"/>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="n"/>
+      <c r="U13" s="4" t="n"/>
+      <c r="V13" s="4" t="n"/>
+      <c r="W13" s="4" t="n"/>
+      <c r="X13" s="4" t="n"/>
+      <c r="Y13" s="4" t="n"/>
+      <c r="Z13" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AA13" s="4" t="n"/>
+      <c r="AB13" s="4" t="n"/>
+      <c r="AC13" s="4" t="n"/>
+      <c r="AD13" s="4" t="n"/>
+      <c r="AE13" s="4" t="n"/>
+      <c r="AF13" s="4" t="n"/>
+      <c r="AG13" s="4" t="n"/>
+      <c r="AH13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AI13" s="4" t="n"/>
+      <c r="AJ13" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+      <c r="AK13" s="4" t="n"/>
+      <c r="AL13" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AM13" s="4" t="n"/>
+      <c r="AN13" s="4" t="n"/>
+      <c r="AO13" s="4" t="n"/>
+      <c r="AP13" s="4" t="n"/>
+      <c r="AQ13" s="3" t="inlineStr">
+        <is>
+          <t>Garde chir</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Martine</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="W14" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AE14" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AF14" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AG14" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AK14" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AL14" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AM14" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AN14" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AO14" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AQ14" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="n"/>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="n"/>
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4" t="n"/>
+      <c r="O15" s="4" t="n"/>
+      <c r="P15" s="4" t="n"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="n"/>
+      <c r="U15" s="4" t="n"/>
+      <c r="V15" s="4" t="n"/>
+      <c r="W15" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="X15" s="4" t="n"/>
+      <c r="Y15" s="4" t="n"/>
+      <c r="Z15" s="4" t="n"/>
+      <c r="AA15" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AB15" s="4" t="n"/>
+      <c r="AC15" s="4" t="n"/>
+      <c r="AD15" s="4" t="n"/>
+      <c r="AE15" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AF15" s="4" t="n"/>
+      <c r="AG15" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AH15" s="4" t="n"/>
+      <c r="AI15" s="4" t="n"/>
+      <c r="AJ15" s="4" t="n"/>
+      <c r="AK15" s="4" t="n"/>
+      <c r="AL15" s="4" t="n"/>
+      <c r="AM15" s="4" t="n"/>
+      <c r="AN15" s="4" t="n"/>
+      <c r="AO15" s="4" t="n"/>
+      <c r="AP15" s="4" t="n"/>
+      <c r="AQ15" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Josselin</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="M16" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="R16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="V16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="W16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="X16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="Y16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="Z16" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AC16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AD16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AE16" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AF16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AG16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AH16" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AJ16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AL16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AN16" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="n"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+      <c r="E17" s="4" t="n"/>
+      <c r="F17" s="4" t="n"/>
+      <c r="G17" s="4" t="n"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
+      <c r="K17" s="4" t="n"/>
+      <c r="L17" s="4" t="n"/>
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4" t="n"/>
+      <c r="Q17" s="4" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="n"/>
+      <c r="T17" s="4" t="n"/>
+      <c r="U17" s="4" t="n"/>
+      <c r="V17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="W17" s="4" t="n"/>
+      <c r="X17" s="4" t="n"/>
+      <c r="Y17" s="4" t="n"/>
+      <c r="Z17" s="4" t="n"/>
+      <c r="AA17" s="4" t="n"/>
+      <c r="AB17" s="4" t="n"/>
+      <c r="AC17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AD17" s="4" t="n"/>
+      <c r="AE17" s="4" t="n"/>
+      <c r="AF17" s="4" t="n"/>
+      <c r="AG17" s="4" t="n"/>
+      <c r="AH17" s="4" t="n"/>
+      <c r="AI17" s="4" t="n"/>
+      <c r="AJ17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AK17" s="4" t="n"/>
+      <c r="AL17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AM17" s="4" t="n"/>
+      <c r="AN17" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AO17" s="4" t="n"/>
+      <c r="AP17" s="4" t="n"/>
+      <c r="AQ17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Martine</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="X18" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="Y18" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="Z18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AA18" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AD18" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AE18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AF18" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AG18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AH18" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AI18" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AK18" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AO18" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="n"/>
+      <c r="B19" s="4" t="n"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="n"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n"/>
+      <c r="G19" s="4" t="n"/>
+      <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="n"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4" t="n"/>
+      <c r="O19" s="4" t="n"/>
+      <c r="P19" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="Q19" s="4" t="n"/>
+      <c r="R19" s="4" t="n"/>
+      <c r="S19" s="4" t="n"/>
+      <c r="T19" s="4" t="n"/>
+      <c r="U19" s="4" t="n"/>
+      <c r="V19" s="4" t="n"/>
+      <c r="W19" s="4" t="n"/>
+      <c r="X19" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="Y19" s="4" t="n"/>
+      <c r="Z19" s="4" t="n"/>
+      <c r="AA19" s="4" t="n"/>
+      <c r="AB19" s="4" t="n"/>
+      <c r="AC19" s="4" t="n"/>
+      <c r="AD19" s="4" t="n"/>
+      <c r="AE19" s="4" t="n"/>
+      <c r="AF19" s="4" t="n"/>
+      <c r="AG19" s="4" t="n"/>
+      <c r="AH19" s="4" t="n"/>
+      <c r="AI19" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AJ19" s="4" t="n"/>
+      <c r="AK19" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AL19" s="4" t="n"/>
+      <c r="AM19" s="4" t="n"/>
+      <c r="AN19" s="4" t="n"/>
+      <c r="AO19" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AP19" s="4" t="n"/>
+      <c r="AQ19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Yoko</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="W20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="X20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AA20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AD20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AE20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AF20" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AG20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AH20" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AK20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AL20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AM20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AN20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="AO20" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="AP20" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+      <c r="E21" s="4" t="n"/>
+      <c r="F21" s="4" t="n"/>
+      <c r="G21" s="4" t="n"/>
+      <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
+      <c r="K21" s="4" t="n"/>
+      <c r="L21" s="4" t="n"/>
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4" t="n"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="P21" s="4" t="n"/>
+      <c r="Q21" s="4" t="n"/>
+      <c r="R21" s="4" t="n"/>
+      <c r="S21" s="4" t="n"/>
+      <c r="T21" s="4" t="n"/>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="V21" s="4" t="n"/>
+      <c r="W21" s="4" t="n"/>
+      <c r="X21" s="4" t="n"/>
+      <c r="Y21" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="Z21" s="4" t="n"/>
+      <c r="AA21" s="4" t="n"/>
+      <c r="AB21" s="4" t="n"/>
+      <c r="AC21" s="4" t="n"/>
+      <c r="AD21" s="4" t="n"/>
+      <c r="AE21" s="4" t="n"/>
+      <c r="AF21" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AG21" s="4" t="n"/>
+      <c r="AH21" s="4" t="n"/>
+      <c r="AI21" s="4" t="n"/>
+      <c r="AJ21" s="4" t="n"/>
+      <c r="AK21" s="4" t="n"/>
+      <c r="AL21" s="4" t="n"/>
+      <c r="AM21" s="4" t="n"/>
+      <c r="AN21" s="4" t="n"/>
+      <c r="AO21" s="4" t="n"/>
+      <c r="AP21" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AQ21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Med3</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="Z22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AB22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AD22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AH22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AK22" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AL22" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AM22" s="5" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="AN22" s="5" t="inlineStr">
+        <is>
+          <t>Consult Van</t>
+        </is>
+      </c>
+      <c r="AO22" s="5" t="inlineStr">
+        <is>
+          <t>Test shift 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="n"/>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4" t="n"/>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Garde mater</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
+      <c r="K23" s="4" t="n"/>
+      <c r="L23" s="4" t="n"/>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="N23" s="4" t="n"/>
+      <c r="O23" s="4" t="n"/>
+      <c r="P23" s="4" t="n"/>
+      <c r="Q23" s="4" t="n"/>
+      <c r="R23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="S23" s="4" t="n"/>
+      <c r="T23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="U23" s="4" t="n"/>
+      <c r="V23" s="4" t="n"/>
+      <c r="W23" s="4" t="n"/>
+      <c r="X23" s="4" t="n"/>
+      <c r="Y23" s="4" t="n"/>
+      <c r="Z23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AA23" s="4" t="n"/>
+      <c r="AB23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AC23" s="4" t="n"/>
+      <c r="AD23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AE23" s="4" t="n"/>
+      <c r="AF23" s="4" t="n"/>
+      <c r="AG23" s="4" t="n"/>
+      <c r="AH23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AI23" s="4" t="n"/>
+      <c r="AJ23" s="4" t="n"/>
+      <c r="AK23" s="4" t="n"/>
+      <c r="AL23" s="4" t="n"/>
+      <c r="AM23" s="3" t="inlineStr">
+        <is>
+          <t>Duty recuperation</t>
+        </is>
+      </c>
+      <c r="AN23" s="4" t="n"/>
+      <c r="AO23" s="4" t="n"/>
+      <c r="AP23" s="4" t="n"/>
+      <c r="AQ23" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A14:A15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>